<commit_message>
Added Additional records 3A tables and 4A inserts
</commit_message>
<xml_diff>
--- a/Rhoden_3A_tables.xlsx
+++ b/Rhoden_3A_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aspennerhoden\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DEDE084-A7E5-430A-AAC0-CF7352962A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F65AEF19-5EB3-4ADA-B562-BC337AA3B3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{FD6B9BBC-4BE4-42A9-BEF2-E36236DB053C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{FD6B9BBC-4BE4-42A9-BEF2-E36236DB053C}"/>
   </bookViews>
   <sheets>
     <sheet name="DogOwner" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="130">
   <si>
     <t>owner_id</t>
   </si>
@@ -319,13 +319,124 @@
   </si>
   <si>
     <t>None</t>
+  </si>
+  <si>
+    <t>Chris</t>
+  </si>
+  <si>
+    <t>Maya</t>
+  </si>
+  <si>
+    <t>516-555-1111</t>
+  </si>
+  <si>
+    <t>718-555-2222</t>
+  </si>
+  <si>
+    <t>3:00PM</t>
+  </si>
+  <si>
+    <t>Eisen Hower Park</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>Zelle</t>
+  </si>
+  <si>
+    <t>Rocky</t>
+  </si>
+  <si>
+    <t>Coco</t>
+  </si>
+  <si>
+    <t>Daisy</t>
+  </si>
+  <si>
+    <t>Milo</t>
+  </si>
+  <si>
+    <t>Sadie</t>
+  </si>
+  <si>
+    <t>Boxer</t>
+  </si>
+  <si>
+    <t>Shih Tzu</t>
+  </si>
+  <si>
+    <t>Labrador Retriever</t>
+  </si>
+  <si>
+    <t>Yorkie</t>
+  </si>
+  <si>
+    <t>Cocker Spaniel</t>
+  </si>
+  <si>
+    <t>Ear infection</t>
+  </si>
+  <si>
+    <t>Skin Allergies</t>
+  </si>
+  <si>
+    <t>Nia</t>
+  </si>
+  <si>
+    <t>Jordan</t>
+  </si>
+  <si>
+    <t>Ava</t>
+  </si>
+  <si>
+    <t>Malik</t>
+  </si>
+  <si>
+    <t>Brianna</t>
+  </si>
+  <si>
+    <t>Ethan</t>
+  </si>
+  <si>
+    <t>Kayla</t>
+  </si>
+  <si>
+    <t>Noah</t>
+  </si>
+  <si>
+    <t>347-555-2101</t>
+  </si>
+  <si>
+    <t>718-555-2102</t>
+  </si>
+  <si>
+    <t>516-555-2103</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 929-555-2104</t>
+  </si>
+  <si>
+    <t>646-555-2105</t>
+  </si>
+  <si>
+    <t>212-555-2106</t>
+  </si>
+  <si>
+    <t>917-555-2107</t>
+  </si>
+  <si>
+    <t>347-555-2108</t>
+  </si>
+  <si>
+    <t>Central Park</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -337,6 +448,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -375,13 +492,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -950,11 +1068,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3A54B52-F4AE-4F9E-8899-CA7F2D9555C8}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="9.36328125" customWidth="1"/>
-    <col min="3" max="3" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.36328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.26953125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1112,6 +1230,136 @@
       </c>
       <c r="H6">
         <v>271</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>1035</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7">
+        <v>62</v>
+      </c>
+      <c r="G7" t="s">
+        <v>92</v>
+      </c>
+      <c r="H7">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>1036</v>
+      </c>
+      <c r="B8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8">
+        <v>14.2</v>
+      </c>
+      <c r="G8" t="s">
+        <v>112</v>
+      </c>
+      <c r="H8">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>1037</v>
+      </c>
+      <c r="B9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9" t="s">
+        <v>88</v>
+      </c>
+      <c r="F9">
+        <v>58.5</v>
+      </c>
+      <c r="G9" t="s">
+        <v>92</v>
+      </c>
+      <c r="H9">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>1038</v>
+      </c>
+      <c r="B10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="G10" t="s">
+        <v>33</v>
+      </c>
+      <c r="H10">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>1039</v>
+      </c>
+      <c r="B11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D11">
+        <v>6</v>
+      </c>
+      <c r="E11" t="s">
+        <v>89</v>
+      </c>
+      <c r="F11">
+        <v>24.6</v>
+      </c>
+      <c r="G11" t="s">
+        <v>111</v>
+      </c>
+      <c r="H11">
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -1121,7 +1369,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A0E794C-2235-46C4-9772-B424D0E56BE0}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="11.54296875" customWidth="1"/>
@@ -1150,19 +1398,130 @@
         <v>35</v>
       </c>
     </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>501</v>
+      </c>
+      <c r="B3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>233</v>
+      </c>
+      <c r="B4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>234</v>
+      </c>
+      <c r="B5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>235</v>
+      </c>
+      <c r="B6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>236</v>
+      </c>
+      <c r="B7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>237</v>
+      </c>
+      <c r="B8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>238</v>
+      </c>
+      <c r="B9" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>239</v>
+      </c>
+      <c r="B10" t="s">
+        <v>118</v>
+      </c>
+      <c r="C10" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>240</v>
+      </c>
+      <c r="B11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>241</v>
+      </c>
+      <c r="B12" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" t="s">
+        <v>128</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A1B37E1-1F18-4351-8A29-176BB9CCF4CB}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="9.26953125" customWidth="1"/>
-    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
@@ -1198,8 +1557,8 @@
       <c r="B2" s="4">
         <v>46129</v>
       </c>
-      <c r="C2" s="5">
-        <v>0.125</v>
+      <c r="C2" s="5" t="s">
+        <v>97</v>
       </c>
       <c r="D2">
         <v>30</v>
@@ -1214,7 +1573,243 @@
         <v>1030</v>
       </c>
       <c r="H2">
-        <v>267</v>
+        <v>233</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>88</v>
+      </c>
+      <c r="B3" s="4">
+        <v>46130</v>
+      </c>
+      <c r="C3" s="6">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D3">
+        <v>30</v>
+      </c>
+      <c r="E3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3">
+        <v>1031</v>
+      </c>
+      <c r="H3">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>89</v>
+      </c>
+      <c r="B4" s="4">
+        <v>46131</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D4">
+        <v>45</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4">
+        <v>1032</v>
+      </c>
+      <c r="H4">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>90</v>
+      </c>
+      <c r="B5" s="4">
+        <v>46132</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5">
+        <v>1033</v>
+      </c>
+      <c r="H5">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>91</v>
+      </c>
+      <c r="B6" s="4">
+        <v>46132</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="E6" t="s">
+        <v>98</v>
+      </c>
+      <c r="F6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6">
+        <v>1034</v>
+      </c>
+      <c r="H6">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>92</v>
+      </c>
+      <c r="B7" s="4">
+        <v>46133</v>
+      </c>
+      <c r="C7" s="6">
+        <v>0.375</v>
+      </c>
+      <c r="E7" t="s">
+        <v>129</v>
+      </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7">
+        <v>1035</v>
+      </c>
+      <c r="H7">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>93</v>
+      </c>
+      <c r="B8" s="4">
+        <v>46133</v>
+      </c>
+      <c r="C8" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8">
+        <v>1036</v>
+      </c>
+      <c r="H8">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>94</v>
+      </c>
+      <c r="B9" s="4">
+        <v>46134</v>
+      </c>
+      <c r="C9" s="6">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9">
+        <v>1037</v>
+      </c>
+      <c r="H9">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>95</v>
+      </c>
+      <c r="B10" s="4">
+        <v>46134</v>
+      </c>
+      <c r="C10" s="6">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="E10" t="s">
+        <v>129</v>
+      </c>
+      <c r="F10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10">
+        <v>1038</v>
+      </c>
+      <c r="H10">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>96</v>
+      </c>
+      <c r="B11" s="4">
+        <v>46135</v>
+      </c>
+      <c r="C11" s="6">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" t="s">
+        <v>37</v>
+      </c>
+      <c r="G11">
+        <v>1039</v>
+      </c>
+      <c r="H11">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>97</v>
+      </c>
+      <c r="B12" s="4">
+        <v>46135</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="E12" t="s">
+        <v>98</v>
+      </c>
+      <c r="F12" t="s">
+        <v>37</v>
+      </c>
+      <c r="G12">
+        <v>1040</v>
+      </c>
+      <c r="H12">
+        <v>241</v>
       </c>
     </row>
   </sheetData>
@@ -1224,7 +1819,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3ADCD02-AABF-4AEF-A719-CD27902C2258}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.90625" customWidth="1"/>
@@ -1273,6 +1868,206 @@
         <v>267</v>
       </c>
     </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>27</v>
+      </c>
+      <c r="B3">
+        <v>65</v>
+      </c>
+      <c r="C3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D3" s="4">
+        <v>46129</v>
+      </c>
+      <c r="E3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>28</v>
+      </c>
+      <c r="B4">
+        <v>70</v>
+      </c>
+      <c r="C4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D4" s="4">
+        <v>46130</v>
+      </c>
+      <c r="E4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>29</v>
+      </c>
+      <c r="B5">
+        <v>75</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="4">
+        <v>46131</v>
+      </c>
+      <c r="E5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>30</v>
+      </c>
+      <c r="B6">
+        <v>60</v>
+      </c>
+      <c r="C6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D6" s="4">
+        <v>46132</v>
+      </c>
+      <c r="E6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>31</v>
+      </c>
+      <c r="B7">
+        <v>85</v>
+      </c>
+      <c r="C7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D7" s="4">
+        <v>46132</v>
+      </c>
+      <c r="E7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>32</v>
+      </c>
+      <c r="B8">
+        <v>50</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="4">
+        <v>46133</v>
+      </c>
+      <c r="E8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>33</v>
+      </c>
+      <c r="B9">
+        <v>95</v>
+      </c>
+      <c r="C9" t="s">
+        <v>99</v>
+      </c>
+      <c r="D9" s="4">
+        <v>46133</v>
+      </c>
+      <c r="E9" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>34</v>
+      </c>
+      <c r="B10">
+        <v>70</v>
+      </c>
+      <c r="C10" t="s">
+        <v>100</v>
+      </c>
+      <c r="D10" s="4">
+        <v>46134</v>
+      </c>
+      <c r="E10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>35</v>
+      </c>
+      <c r="B11">
+        <v>80</v>
+      </c>
+      <c r="C11" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="4">
+        <v>46134</v>
+      </c>
+      <c r="E11" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>36</v>
+      </c>
+      <c r="B12">
+        <v>65</v>
+      </c>
+      <c r="C12" t="s">
+        <v>99</v>
+      </c>
+      <c r="D12" s="4">
+        <v>46135</v>
+      </c>
+      <c r="E12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12">
+        <v>277</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>